<commit_message>
Fix column widths cut off on Rule of 40 and Magic Number tabs
Caught while opening the workbook to check the Rule of 40 tab: column A
was too narrow for the "Rule of 40 (current quarter)" result label, and
the Magic Number benchmark table's Action column was too narrow for
"Invest cautiously" / "Scale now". Cosmetic only — formulas and values
were already correct — but visible in normal Excel view, not just print.
Re-verified with recalc.py (zero errors) and a rendered PDF preview.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015iFnPUPZY9ogRLiF1pW3WP
</commit_message>
<xml_diff>
--- a/Artifacts/business/saas-growth-efficiency-dashboard.xlsx
+++ b/Artifacts/business/saas-growth-efficiency-dashboard.xlsx
@@ -1366,11 +1366,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="34635909"/>
-        <c:axId val="76095754"/>
+        <c:axId val="28751373"/>
+        <c:axId val="59664438"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="34635909"/>
+        <c:axId val="28751373"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1402,7 +1402,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76095754"/>
+        <c:crossAx val="59664438"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1410,7 +1410,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="76095754"/>
+        <c:axId val="59664438"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1486,7 +1486,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34635909"/>
+        <c:crossAx val="28751373"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1775,11 +1775,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="84652422"/>
-        <c:axId val="61960735"/>
+        <c:axId val="23221431"/>
+        <c:axId val="95595480"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="84652422"/>
+        <c:axId val="23221431"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1811,7 +1811,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61960735"/>
+        <c:crossAx val="95595480"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1819,7 +1819,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61960735"/>
+        <c:axId val="95595480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1895,7 +1895,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84652422"/>
+        <c:crossAx val="23221431"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2101,11 +2101,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="58551823"/>
-        <c:axId val="61862788"/>
+        <c:axId val="39919496"/>
+        <c:axId val="41894354"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="58551823"/>
+        <c:axId val="39919496"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2181,12 +2181,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61862788"/>
+        <c:crossAx val="41894354"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="61862788"/>
+        <c:axId val="41894354"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2262,7 +2262,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58551823"/>
+        <c:crossAx val="39919496"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2660,11 +2660,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="49413187"/>
-        <c:axId val="30312576"/>
+        <c:axId val="70256143"/>
+        <c:axId val="8176527"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="49413187"/>
+        <c:axId val="70256143"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2730,7 +2730,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30312576"/>
+        <c:crossAx val="8176527"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2738,7 +2738,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30312576"/>
+        <c:axId val="8176527"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2814,7 +2814,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49413187"/>
+        <c:crossAx val="70256143"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2876,8 +2876,8 @@
       <xdr:rowOff>101160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>790200</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>967680</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>123120</xdr:rowOff>
     </xdr:to>
@@ -3390,7 +3390,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
   </cols>
@@ -3454,7 +3454,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
@@ -3540,7 +3540,7 @@
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>

</xml_diff>